<commit_message>
v1.4.2: Fix NPT3"/NPT4" thread DB (d2 was incorrectly set equal to d_major)
NPT3": (87.884,85.798,87.884) -> (86.068,83.982,87.884) [ASME B1.20.1 E1]
NPT4": (113.030,110.944,113.030) -> (111.433,109.347,113.030)
d2=d_major caused wrong thread depth in simulation. Updated Excel.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/thread_pass_simulation.xlsx
+++ b/thread_pass_simulation.xlsx
@@ -24011,31 +24011,31 @@
         <v>0.32</v>
       </c>
       <c r="G248" s="2" t="n">
-        <v>1.2698</v>
+        <v>2.1778</v>
       </c>
       <c r="H248" s="2" t="n">
-        <v>1.3198</v>
+        <v>2.2278</v>
       </c>
       <c r="I248" s="2" t="n">
         <v>8</v>
       </c>
       <c r="J248" s="3" t="n">
-        <v>0.5279</v>
+        <v>0.8911</v>
       </c>
       <c r="K248" s="3" t="n">
-        <v>0.2187</v>
+        <v>0.3691</v>
       </c>
       <c r="L248" s="3" t="n">
-        <v>0.1677</v>
+        <v>0.2832</v>
       </c>
       <c r="M248" s="3" t="n">
-        <v>0.1415</v>
+        <v>0.2388</v>
       </c>
       <c r="N248" s="3" t="n">
-        <v>0.1246</v>
+        <v>0.2104</v>
       </c>
       <c r="O248" s="3" t="n">
-        <v>0.08939999999999999</v>
+        <v>0.1852</v>
       </c>
       <c r="P248" s="4" t="n">
         <v>0.05</v>
@@ -24050,28 +24050,28 @@
       <c r="V248" s="5" t="n"/>
       <c r="W248" s="5" t="n"/>
       <c r="X248" s="6" t="n">
-        <v>86.928</v>
+        <v>86.202</v>
       </c>
       <c r="Y248" s="6" t="n">
-        <v>86.491</v>
+        <v>85.464</v>
       </c>
       <c r="Z248" s="6" t="n">
-        <v>86.15600000000001</v>
+        <v>84.898</v>
       </c>
       <c r="AA248" s="6" t="n">
-        <v>85.873</v>
+        <v>84.42</v>
       </c>
       <c r="AB248" s="6" t="n">
-        <v>85.624</v>
+        <v>83.999</v>
       </c>
       <c r="AC248" s="6" t="n">
-        <v>85.44499999999999</v>
+        <v>83.629</v>
       </c>
       <c r="AD248" s="7" t="n">
-        <v>85.345</v>
+        <v>83.529</v>
       </c>
       <c r="AE248" s="7" t="n">
-        <v>85.345</v>
+        <v>83.529</v>
       </c>
       <c r="AF248" s="5" t="n"/>
       <c r="AG248" s="5" t="n"/>
@@ -24106,88 +24106,72 @@
         <v>0.32</v>
       </c>
       <c r="G249" s="2" t="n">
-        <v>2.9935</v>
+        <v>2.0855</v>
       </c>
       <c r="H249" s="2" t="n">
-        <v>3.0435</v>
+        <v>2.1355</v>
       </c>
       <c r="I249" s="2" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="J249" s="3" t="n">
-        <v>0.9525</v>
+        <v>0.8542</v>
       </c>
       <c r="K249" s="3" t="n">
-        <v>0.3945</v>
+        <v>0.3538</v>
       </c>
       <c r="L249" s="3" t="n">
-        <v>0.3028</v>
+        <v>0.2715</v>
       </c>
       <c r="M249" s="3" t="n">
-        <v>0.2552</v>
+        <v>0.2289</v>
       </c>
       <c r="N249" s="3" t="n">
-        <v>0.2249</v>
+        <v>0.2016</v>
       </c>
       <c r="O249" s="3" t="n">
-        <v>0.2032</v>
-      </c>
-      <c r="P249" s="3" t="n">
-        <v>0.187</v>
-      </c>
-      <c r="Q249" s="3" t="n">
-        <v>0.174</v>
-      </c>
-      <c r="R249" s="3" t="n">
-        <v>0.1634</v>
-      </c>
-      <c r="S249" s="3" t="n">
-        <v>0.136</v>
-      </c>
-      <c r="T249" s="4" t="n">
+        <v>0.1755</v>
+      </c>
+      <c r="P249" s="4" t="n">
         <v>0.05</v>
       </c>
-      <c r="U249" s="4" t="n">
+      <c r="Q249" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="R249" s="5" t="n"/>
+      <c r="S249" s="5" t="n"/>
+      <c r="T249" s="5" t="n"/>
+      <c r="U249" s="5" t="n"/>
       <c r="V249" s="5" t="n"/>
       <c r="W249" s="5" t="n"/>
       <c r="X249" s="6" t="n">
-        <v>86.252</v>
+        <v>86.05500000000001</v>
       </c>
       <c r="Y249" s="6" t="n">
-        <v>87.041</v>
+        <v>86.76300000000001</v>
       </c>
       <c r="Z249" s="6" t="n">
-        <v>87.64700000000001</v>
+        <v>87.306</v>
       </c>
       <c r="AA249" s="6" t="n">
-        <v>88.157</v>
+        <v>87.764</v>
       </c>
       <c r="AB249" s="6" t="n">
-        <v>88.607</v>
+        <v>88.167</v>
       </c>
       <c r="AC249" s="6" t="n">
-        <v>89.01300000000001</v>
-      </c>
-      <c r="AD249" s="6" t="n">
-        <v>89.387</v>
-      </c>
-      <c r="AE249" s="6" t="n">
-        <v>89.735</v>
-      </c>
-      <c r="AF249" s="6" t="n">
-        <v>90.062</v>
-      </c>
-      <c r="AG249" s="6" t="n">
-        <v>90.334</v>
-      </c>
-      <c r="AH249" s="7" t="n">
-        <v>90.434</v>
-      </c>
-      <c r="AI249" s="7" t="n">
-        <v>90.434</v>
-      </c>
+        <v>88.518</v>
+      </c>
+      <c r="AD249" s="7" t="n">
+        <v>88.61799999999999</v>
+      </c>
+      <c r="AE249" s="7" t="n">
+        <v>88.61799999999999</v>
+      </c>
+      <c r="AF249" s="5" t="n"/>
+      <c r="AG249" s="5" t="n"/>
+      <c r="AH249" s="5" t="n"/>
+      <c r="AI249" s="5" t="n"/>
       <c r="AJ249" s="5" t="n"/>
       <c r="AK249" s="5" t="n"/>
     </row>
@@ -24217,31 +24201,31 @@
         <v>0.32</v>
       </c>
       <c r="G250" s="2" t="n">
-        <v>1.2785</v>
+        <v>2.077</v>
       </c>
       <c r="H250" s="2" t="n">
-        <v>1.3285</v>
+        <v>2.127</v>
       </c>
       <c r="I250" s="2" t="n">
         <v>8</v>
       </c>
       <c r="J250" s="3" t="n">
-        <v>0.5314</v>
+        <v>0.8508</v>
       </c>
       <c r="K250" s="3" t="n">
-        <v>0.2201</v>
+        <v>0.3524</v>
       </c>
       <c r="L250" s="3" t="n">
-        <v>0.1689</v>
+        <v>0.2704</v>
       </c>
       <c r="M250" s="3" t="n">
-        <v>0.1424</v>
+        <v>0.228</v>
       </c>
       <c r="N250" s="3" t="n">
-        <v>0.1254</v>
+        <v>0.2008</v>
       </c>
       <c r="O250" s="3" t="n">
-        <v>0.09030000000000001</v>
+        <v>0.1746</v>
       </c>
       <c r="P250" s="4" t="n">
         <v>0.05</v>
@@ -24256,28 +24240,28 @@
       <c r="V250" s="5" t="n"/>
       <c r="W250" s="5" t="n"/>
       <c r="X250" s="6" t="n">
-        <v>112.067</v>
+        <v>111.428</v>
       </c>
       <c r="Y250" s="6" t="n">
-        <v>111.627</v>
+        <v>110.723</v>
       </c>
       <c r="Z250" s="6" t="n">
-        <v>111.289</v>
+        <v>110.182</v>
       </c>
       <c r="AA250" s="6" t="n">
-        <v>111.004</v>
+        <v>109.726</v>
       </c>
       <c r="AB250" s="6" t="n">
-        <v>110.753</v>
+        <v>109.324</v>
       </c>
       <c r="AC250" s="6" t="n">
-        <v>110.572</v>
+        <v>108.975</v>
       </c>
       <c r="AD250" s="7" t="n">
-        <v>110.472</v>
+        <v>108.875</v>
       </c>
       <c r="AE250" s="7" t="n">
-        <v>110.472</v>
+        <v>108.875</v>
       </c>
       <c r="AF250" s="5" t="n"/>
       <c r="AG250" s="5" t="n"/>
@@ -24312,88 +24296,72 @@
         <v>0.32</v>
       </c>
       <c r="G251" s="2" t="n">
-        <v>3.0045</v>
+        <v>2.206</v>
       </c>
       <c r="H251" s="2" t="n">
-        <v>3.0545</v>
+        <v>2.256</v>
       </c>
       <c r="I251" s="2" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="J251" s="3" t="n">
-        <v>0.9525</v>
+        <v>0.9024</v>
       </c>
       <c r="K251" s="3" t="n">
-        <v>0.3945</v>
+        <v>0.3738</v>
       </c>
       <c r="L251" s="3" t="n">
-        <v>0.3028</v>
+        <v>0.2868</v>
       </c>
       <c r="M251" s="3" t="n">
-        <v>0.2552</v>
+        <v>0.2418</v>
       </c>
       <c r="N251" s="3" t="n">
-        <v>0.2249</v>
+        <v>0.213</v>
       </c>
       <c r="O251" s="3" t="n">
-        <v>0.2032</v>
-      </c>
-      <c r="P251" s="3" t="n">
-        <v>0.187</v>
-      </c>
-      <c r="Q251" s="3" t="n">
-        <v>0.174</v>
-      </c>
-      <c r="R251" s="3" t="n">
-        <v>0.1634</v>
-      </c>
-      <c r="S251" s="3" t="n">
-        <v>0.147</v>
-      </c>
-      <c r="T251" s="4" t="n">
+        <v>0.1882</v>
+      </c>
+      <c r="P251" s="4" t="n">
         <v>0.05</v>
       </c>
-      <c r="U251" s="4" t="n">
+      <c r="Q251" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="R251" s="5" t="n"/>
+      <c r="S251" s="5" t="n"/>
+      <c r="T251" s="5" t="n"/>
+      <c r="U251" s="5" t="n"/>
       <c r="V251" s="5" t="n"/>
       <c r="W251" s="5" t="n"/>
       <c r="X251" s="6" t="n">
-        <v>111.398</v>
+        <v>111.298</v>
       </c>
       <c r="Y251" s="6" t="n">
-        <v>112.187</v>
+        <v>112.046</v>
       </c>
       <c r="Z251" s="6" t="n">
-        <v>112.793</v>
+        <v>112.62</v>
       </c>
       <c r="AA251" s="6" t="n">
-        <v>113.303</v>
+        <v>113.104</v>
       </c>
       <c r="AB251" s="6" t="n">
-        <v>113.753</v>
+        <v>113.53</v>
       </c>
       <c r="AC251" s="6" t="n">
-        <v>114.159</v>
-      </c>
-      <c r="AD251" s="6" t="n">
-        <v>114.533</v>
-      </c>
-      <c r="AE251" s="6" t="n">
-        <v>114.881</v>
-      </c>
-      <c r="AF251" s="6" t="n">
-        <v>115.208</v>
-      </c>
-      <c r="AG251" s="6" t="n">
-        <v>115.502</v>
-      </c>
-      <c r="AH251" s="7" t="n">
-        <v>115.602</v>
-      </c>
-      <c r="AI251" s="7" t="n">
-        <v>115.602</v>
-      </c>
+        <v>113.906</v>
+      </c>
+      <c r="AD251" s="7" t="n">
+        <v>114.006</v>
+      </c>
+      <c r="AE251" s="7" t="n">
+        <v>114.006</v>
+      </c>
+      <c r="AF251" s="5" t="n"/>
+      <c r="AG251" s="5" t="n"/>
+      <c r="AH251" s="5" t="n"/>
+      <c r="AI251" s="5" t="n"/>
       <c r="AJ251" s="5" t="n"/>
       <c r="AK251" s="5" t="n"/>
     </row>
@@ -55211,10 +55179,10 @@
         <v>0.32</v>
       </c>
       <c r="G248" s="2" t="n">
-        <v>1.2698</v>
+        <v>2.1778</v>
       </c>
       <c r="H248" s="2" t="n">
-        <v>1.3198</v>
+        <v>2.2278</v>
       </c>
       <c r="I248" s="2" t="n">
         <v>0.9525</v>
@@ -55223,31 +55191,35 @@
         <v>0.1</v>
       </c>
       <c r="K248" s="2" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="L248" s="3" t="n">
         <v>0.4763</v>
       </c>
       <c r="M248" s="3" t="n">
-        <v>0.3172</v>
+        <v>0.4763</v>
       </c>
       <c r="N248" s="3" t="n">
+        <v>0.4763</v>
+      </c>
+      <c r="O248" s="3" t="n">
+        <v>0.2727</v>
+      </c>
+      <c r="P248" s="3" t="n">
         <v>0.2381</v>
       </c>
-      <c r="O248" s="3" t="n">
+      <c r="Q248" s="3" t="n">
         <v>0.1191</v>
       </c>
-      <c r="P248" s="3" t="n">
+      <c r="R248" s="3" t="n">
         <v>0.0595</v>
       </c>
-      <c r="Q248" s="3" t="n">
+      <c r="S248" s="3" t="n">
         <v>0.0595</v>
       </c>
-      <c r="R248" s="3" t="n">
+      <c r="T248" s="3" t="n">
         <v>0.0501</v>
       </c>
-      <c r="S248" s="5" t="n"/>
-      <c r="T248" s="5" t="n"/>
       <c r="U248" s="5" t="n"/>
       <c r="V248" s="5" t="n"/>
       <c r="W248" s="5" t="n"/>
@@ -55257,25 +55229,29 @@
         <v>87.03100000000001</v>
       </c>
       <c r="AA248" s="6" t="n">
-        <v>86.39700000000001</v>
+        <v>86.078</v>
       </c>
       <c r="AB248" s="6" t="n">
-        <v>85.92100000000001</v>
+        <v>85.125</v>
       </c>
       <c r="AC248" s="6" t="n">
-        <v>85.68300000000001</v>
+        <v>84.58</v>
       </c>
       <c r="AD248" s="6" t="n">
-        <v>85.56399999999999</v>
+        <v>84.104</v>
       </c>
       <c r="AE248" s="6" t="n">
-        <v>85.44499999999999</v>
+        <v>83.866</v>
       </c>
       <c r="AF248" s="6" t="n">
-        <v>85.345</v>
-      </c>
-      <c r="AG248" s="5" t="n"/>
-      <c r="AH248" s="5" t="n"/>
+        <v>83.747</v>
+      </c>
+      <c r="AG248" s="6" t="n">
+        <v>83.628</v>
+      </c>
+      <c r="AH248" s="6" t="n">
+        <v>83.52800000000001</v>
+      </c>
       <c r="AI248" s="5" t="n"/>
       <c r="AJ248" s="5" t="n"/>
       <c r="AK248" s="5" t="n"/>
@@ -55308,10 +55284,10 @@
         <v>0.32</v>
       </c>
       <c r="G249" s="2" t="n">
-        <v>2.9935</v>
+        <v>2.0855</v>
       </c>
       <c r="H249" s="2" t="n">
-        <v>3.0435</v>
+        <v>2.1355</v>
       </c>
       <c r="I249" s="2" t="n">
         <v>0.9525</v>
@@ -55320,7 +55296,7 @@
         <v>0.1</v>
       </c>
       <c r="K249" s="2" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="L249" s="3" t="n">
         <v>0.4763</v>
@@ -55332,29 +55308,25 @@
         <v>0.4763</v>
       </c>
       <c r="O249" s="3" t="n">
-        <v>0.4763</v>
+        <v>0.1804</v>
       </c>
       <c r="P249" s="3" t="n">
-        <v>0.4763</v>
+        <v>0.2381</v>
       </c>
       <c r="Q249" s="3" t="n">
-        <v>0.136</v>
+        <v>0.1191</v>
       </c>
       <c r="R249" s="3" t="n">
-        <v>0.2381</v>
+        <v>0.0595</v>
       </c>
       <c r="S249" s="3" t="n">
-        <v>0.1191</v>
+        <v>0.0595</v>
       </c>
       <c r="T249" s="3" t="n">
-        <v>0.0595</v>
-      </c>
-      <c r="U249" s="3" t="n">
-        <v>0.0595</v>
-      </c>
-      <c r="V249" s="3" t="n">
-        <v>0.05</v>
-      </c>
+        <v>0.0501</v>
+      </c>
+      <c r="U249" s="5" t="n"/>
+      <c r="V249" s="5" t="n"/>
       <c r="W249" s="5" t="n"/>
       <c r="X249" s="5" t="n"/>
       <c r="Y249" s="5" t="n"/>
@@ -55368,29 +55340,25 @@
         <v>87.206</v>
       </c>
       <c r="AC249" s="6" t="n">
-        <v>88.15900000000001</v>
+        <v>87.56699999999999</v>
       </c>
       <c r="AD249" s="6" t="n">
-        <v>89.11199999999999</v>
+        <v>88.04300000000001</v>
       </c>
       <c r="AE249" s="6" t="n">
-        <v>89.384</v>
+        <v>88.28100000000001</v>
       </c>
       <c r="AF249" s="6" t="n">
-        <v>89.86</v>
+        <v>88.40000000000001</v>
       </c>
       <c r="AG249" s="6" t="n">
-        <v>90.098</v>
+        <v>88.51900000000001</v>
       </c>
       <c r="AH249" s="6" t="n">
-        <v>90.217</v>
-      </c>
-      <c r="AI249" s="6" t="n">
-        <v>90.336</v>
-      </c>
-      <c r="AJ249" s="6" t="n">
-        <v>90.43600000000001</v>
-      </c>
+        <v>88.619</v>
+      </c>
+      <c r="AI249" s="5" t="n"/>
+      <c r="AJ249" s="5" t="n"/>
       <c r="AK249" s="5" t="n"/>
       <c r="AL249" s="5" t="n"/>
       <c r="AM249" s="5" t="n"/>
@@ -55421,10 +55389,10 @@
         <v>0.32</v>
       </c>
       <c r="G250" s="2" t="n">
-        <v>1.2785</v>
+        <v>2.077</v>
       </c>
       <c r="H250" s="2" t="n">
-        <v>1.3285</v>
+        <v>2.127</v>
       </c>
       <c r="I250" s="2" t="n">
         <v>0.9525</v>
@@ -55433,31 +55401,35 @@
         <v>0.1</v>
       </c>
       <c r="K250" s="2" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="L250" s="3" t="n">
         <v>0.4763</v>
       </c>
       <c r="M250" s="3" t="n">
-        <v>0.3259</v>
+        <v>0.4763</v>
       </c>
       <c r="N250" s="3" t="n">
+        <v>0.4763</v>
+      </c>
+      <c r="O250" s="3" t="n">
+        <v>0.1719</v>
+      </c>
+      <c r="P250" s="3" t="n">
         <v>0.2381</v>
       </c>
-      <c r="O250" s="3" t="n">
+      <c r="Q250" s="3" t="n">
         <v>0.1191</v>
       </c>
-      <c r="P250" s="3" t="n">
+      <c r="R250" s="3" t="n">
         <v>0.0595</v>
       </c>
-      <c r="Q250" s="3" t="n">
+      <c r="S250" s="3" t="n">
         <v>0.0595</v>
       </c>
-      <c r="R250" s="3" t="n">
+      <c r="T250" s="3" t="n">
         <v>0.0501</v>
       </c>
-      <c r="S250" s="5" t="n"/>
-      <c r="T250" s="5" t="n"/>
       <c r="U250" s="5" t="n"/>
       <c r="V250" s="5" t="n"/>
       <c r="W250" s="5" t="n"/>
@@ -55467,25 +55439,29 @@
         <v>112.177</v>
       </c>
       <c r="AA250" s="6" t="n">
-        <v>111.525</v>
+        <v>111.224</v>
       </c>
       <c r="AB250" s="6" t="n">
-        <v>111.049</v>
+        <v>110.271</v>
       </c>
       <c r="AC250" s="6" t="n">
-        <v>110.811</v>
+        <v>109.927</v>
       </c>
       <c r="AD250" s="6" t="n">
-        <v>110.692</v>
+        <v>109.451</v>
       </c>
       <c r="AE250" s="6" t="n">
-        <v>110.573</v>
+        <v>109.213</v>
       </c>
       <c r="AF250" s="6" t="n">
-        <v>110.473</v>
-      </c>
-      <c r="AG250" s="5" t="n"/>
-      <c r="AH250" s="5" t="n"/>
+        <v>109.094</v>
+      </c>
+      <c r="AG250" s="6" t="n">
+        <v>108.975</v>
+      </c>
+      <c r="AH250" s="6" t="n">
+        <v>108.875</v>
+      </c>
       <c r="AI250" s="5" t="n"/>
       <c r="AJ250" s="5" t="n"/>
       <c r="AK250" s="5" t="n"/>
@@ -55518,10 +55494,10 @@
         <v>0.32</v>
       </c>
       <c r="G251" s="2" t="n">
-        <v>3.0045</v>
+        <v>2.206</v>
       </c>
       <c r="H251" s="2" t="n">
-        <v>3.0545</v>
+        <v>2.256</v>
       </c>
       <c r="I251" s="2" t="n">
         <v>0.9525</v>
@@ -55530,7 +55506,7 @@
         <v>0.1</v>
       </c>
       <c r="K251" s="2" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="L251" s="3" t="n">
         <v>0.4763</v>
@@ -55542,29 +55518,25 @@
         <v>0.4763</v>
       </c>
       <c r="O251" s="3" t="n">
-        <v>0.4763</v>
+        <v>0.3009</v>
       </c>
       <c r="P251" s="3" t="n">
-        <v>0.4763</v>
+        <v>0.2381</v>
       </c>
       <c r="Q251" s="3" t="n">
-        <v>0.147</v>
+        <v>0.1191</v>
       </c>
       <c r="R251" s="3" t="n">
-        <v>0.2381</v>
+        <v>0.0595</v>
       </c>
       <c r="S251" s="3" t="n">
-        <v>0.1191</v>
+        <v>0.0595</v>
       </c>
       <c r="T251" s="3" t="n">
-        <v>0.0595</v>
-      </c>
-      <c r="U251" s="3" t="n">
-        <v>0.0595</v>
-      </c>
-      <c r="V251" s="3" t="n">
-        <v>0.05</v>
-      </c>
+        <v>0.0501</v>
+      </c>
+      <c r="U251" s="5" t="n"/>
+      <c r="V251" s="5" t="n"/>
       <c r="W251" s="5" t="n"/>
       <c r="X251" s="5" t="n"/>
       <c r="Y251" s="5" t="n"/>
@@ -55578,29 +55550,25 @@
         <v>112.352</v>
       </c>
       <c r="AC251" s="6" t="n">
-        <v>113.305</v>
+        <v>112.954</v>
       </c>
       <c r="AD251" s="6" t="n">
-        <v>114.258</v>
+        <v>113.43</v>
       </c>
       <c r="AE251" s="6" t="n">
-        <v>114.552</v>
+        <v>113.668</v>
       </c>
       <c r="AF251" s="6" t="n">
-        <v>115.028</v>
+        <v>113.787</v>
       </c>
       <c r="AG251" s="6" t="n">
-        <v>115.266</v>
+        <v>113.906</v>
       </c>
       <c r="AH251" s="6" t="n">
-        <v>115.385</v>
-      </c>
-      <c r="AI251" s="6" t="n">
-        <v>115.504</v>
-      </c>
-      <c r="AJ251" s="6" t="n">
-        <v>115.604</v>
-      </c>
+        <v>114.006</v>
+      </c>
+      <c r="AI251" s="5" t="n"/>
+      <c r="AJ251" s="5" t="n"/>
       <c r="AK251" s="5" t="n"/>
       <c r="AL251" s="5" t="n"/>
       <c r="AM251" s="5" t="n"/>

</xml_diff>